<commit_message>
feat: Day 2 of world cup
</commit_message>
<xml_diff>
--- a/Projects/FIFACompetition/WorldCup2026/data/World Cup 2026.xlsx
+++ b/Projects/FIFACompetition/WorldCup2026/data/World Cup 2026.xlsx
@@ -8,9 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roman\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2B2BE3-B351-4A91-9F4E-4A2A5E281C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F76DCD-2F2C-43CE-A376-696E3435EFD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EB416841-6D47-41C4-90DD-B677D38E65E5}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="6216" activeTab="1" xr2:uid="{FA6ECF04-EE65-4057-9D05-B2AD136BFF74}"/>
+    <workbookView xWindow="11424" yWindow="6120" windowWidth="11712" windowHeight="6216" activeTab="2" xr2:uid="{2CE22ED6-905D-4770-8C84-A6921D1589AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Squads" sheetId="1" r:id="rId1"/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="321">
   <si>
     <t>ID</t>
   </si>
@@ -170,12 +171,6 @@
     <t>squad_id</t>
   </si>
   <si>
-    <t>WC-2026-016</t>
-  </si>
-  <si>
-    <t>WC-2026-001</t>
-  </si>
-  <si>
     <t>WC-2026-002</t>
   </si>
   <si>
@@ -194,9 +189,6 @@
     <t>WC-2026-007</t>
   </si>
   <si>
-    <t>WC-2026-008</t>
-  </si>
-  <si>
     <t>WC-2026-009</t>
   </si>
   <si>
@@ -224,16 +216,781 @@
     <t>WC-2026-018</t>
   </si>
   <si>
-    <t>WC-2026-019</t>
-  </si>
-  <si>
-    <t>WC-2026-020</t>
-  </si>
-  <si>
-    <t>WC-2026-021</t>
-  </si>
-  <si>
     <t>WC-2026-022</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>Guillermo</t>
+  </si>
+  <si>
+    <t>Israel</t>
+  </si>
+  <si>
+    <t>Brian</t>
+  </si>
+  <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>Roberto</t>
+  </si>
+  <si>
+    <t>Ronwen</t>
+  </si>
+  <si>
+    <t>Aubrey</t>
+  </si>
+  <si>
+    <t>Khuliso</t>
+  </si>
+  <si>
+    <t>Nkosinathi</t>
+  </si>
+  <si>
+    <t>Khulumani</t>
+  </si>
+  <si>
+    <t>Sphephelo</t>
+  </si>
+  <si>
+    <t>Themba</t>
+  </si>
+  <si>
+    <t>Relebohile</t>
+  </si>
+  <si>
+    <t>Oswin</t>
+  </si>
+  <si>
+    <t>Lyle</t>
+  </si>
+  <si>
+    <t>Lira</t>
+  </si>
+  <si>
+    <t>Ochoa</t>
+  </si>
+  <si>
+    <t>Gallardo</t>
+  </si>
+  <si>
+    <t>Montes</t>
+  </si>
+  <si>
+    <t>Reyes</t>
+  </si>
+  <si>
+    <t>Fidalgo</t>
+  </si>
+  <si>
+    <t>Williams</t>
+  </si>
+  <si>
+    <t>Modiba</t>
+  </si>
+  <si>
+    <t>Mudau</t>
+  </si>
+  <si>
+    <t>Sibisi</t>
+  </si>
+  <si>
+    <t>Sithole</t>
+  </si>
+  <si>
+    <t>Zwane</t>
+  </si>
+  <si>
+    <t>Mofokeng</t>
+  </si>
+  <si>
+    <t>Foster</t>
+  </si>
+  <si>
+    <t>Jesus</t>
+  </si>
+  <si>
+    <t>Johan</t>
+  </si>
+  <si>
+    <t>Teboho</t>
+  </si>
+  <si>
+    <t>Vasquez</t>
+  </si>
+  <si>
+    <t>Cesar</t>
+  </si>
+  <si>
+    <t>Erik</t>
+  </si>
+  <si>
+    <t>Alvaro</t>
+  </si>
+  <si>
+    <t>Guttierez</t>
+  </si>
+  <si>
+    <t>Gimenez</t>
+  </si>
+  <si>
+    <t>Raul</t>
+  </si>
+  <si>
+    <t>Jimenez</t>
+  </si>
+  <si>
+    <t>Alverdo</t>
+  </si>
+  <si>
+    <t>Ndimane</t>
+  </si>
+  <si>
+    <t>Mokoena</t>
+  </si>
+  <si>
+    <t>Apollis</t>
+  </si>
+  <si>
+    <t>Rangel</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ra%C3%BAl_Rangel_(footballer)</t>
+  </si>
+  <si>
+    <t>Julian</t>
+  </si>
+  <si>
+    <t>Quinones</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Juli%C3%A1n_Qui%C3%B1ones</t>
+  </si>
+  <si>
+    <t>Iqraam</t>
+  </si>
+  <si>
+    <t>Rayners</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Iqraam_Rayners</t>
+  </si>
+  <si>
+    <t>Jayden</t>
+  </si>
+  <si>
+    <t>Adams</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Jayden_Adams</t>
+  </si>
+  <si>
+    <t>Mbekezeli</t>
+  </si>
+  <si>
+    <t>Mbokazi</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Mbekezeli_Mbokazi</t>
+  </si>
+  <si>
+    <t>Ime</t>
+  </si>
+  <si>
+    <t>Okon</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ime_Okon</t>
+  </si>
+  <si>
+    <t>Kim</t>
+  </si>
+  <si>
+    <t>Seung-gyu</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Kim_Seung-gyu</t>
+  </si>
+  <si>
+    <t>Lee</t>
+  </si>
+  <si>
+    <t>Han-beom</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Lee_Han-beom</t>
+  </si>
+  <si>
+    <t>Min-jae</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Kim_Min-jae_(footballer)</t>
+  </si>
+  <si>
+    <t>Gi-hyuk</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Lee_Gi-hyuk</t>
+  </si>
+  <si>
+    <t>Seol</t>
+  </si>
+  <si>
+    <t>Young-woo</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Seol_Young-woo</t>
+  </si>
+  <si>
+    <t>Hwang</t>
+  </si>
+  <si>
+    <t>In-beom</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Hwang_In-beom</t>
+  </si>
+  <si>
+    <t>Paik</t>
+  </si>
+  <si>
+    <t>Seung-ho</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Paik_Seung-ho</t>
+  </si>
+  <si>
+    <t>Tae-seok</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Lee_Tae-seok</t>
+  </si>
+  <si>
+    <t>Kang-in</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Lee_Kang-in</t>
+  </si>
+  <si>
+    <t>Son</t>
+  </si>
+  <si>
+    <t>Heung-min</t>
+  </si>
+  <si>
+    <t>2010,2014,2018,2022,2026</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Son_Heung-min</t>
+  </si>
+  <si>
+    <t>Jae-sung</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Lee_Jae-sung</t>
+  </si>
+  <si>
+    <t>Pavel</t>
+  </si>
+  <si>
+    <t>Sulc</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Pavel_%C5%A0ulc</t>
+  </si>
+  <si>
+    <t>Patrik</t>
+  </si>
+  <si>
+    <t>Schick</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Patrik_Schick</t>
+  </si>
+  <si>
+    <t>Lukas</t>
+  </si>
+  <si>
+    <t>Provod</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Luk%C3%A1%C5%A1_Provod</t>
+  </si>
+  <si>
+    <t>Jaroslav</t>
+  </si>
+  <si>
+    <t>Zeleny</t>
+  </si>
+  <si>
+    <t>https://cs.wikipedia.org/wiki/Jaroslav_Zelen%C3%BD</t>
+  </si>
+  <si>
+    <t>Alexandr</t>
+  </si>
+  <si>
+    <t>Sojka</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Alexandr_Sojka</t>
+  </si>
+  <si>
+    <t>Tomas</t>
+  </si>
+  <si>
+    <t>Soucek</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Tom%C3%A1%C5%A1_Sou%C4%8Dek</t>
+  </si>
+  <si>
+    <t>Vladimir</t>
+  </si>
+  <si>
+    <t>Coufal</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Vladim%C3%ADr_Coufal</t>
+  </si>
+  <si>
+    <t>Ladislav</t>
+  </si>
+  <si>
+    <t>Krejci</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ladislav_Krej%C4%8D%C3%AD_(footballer,_born_1999)</t>
+  </si>
+  <si>
+    <t>Robin</t>
+  </si>
+  <si>
+    <t>Hranac</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Robin_Hran%C3%A1%C4%8D</t>
+  </si>
+  <si>
+    <t>Stephan</t>
+  </si>
+  <si>
+    <t>Chaloupek</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/%C5%A0t%C4%9Bp%C3%A1n_Chaloupek</t>
+  </si>
+  <si>
+    <t>Matej</t>
+  </si>
+  <si>
+    <t>Kovar</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Mat%C4%9Bj_Kov%C3%A1%C5%99</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>Squad agains Czech Republic</t>
+  </si>
+  <si>
+    <t>Czech Republic</t>
+  </si>
+  <si>
+    <t>Squad agains South Korea</t>
+  </si>
+  <si>
+    <t>WC-2026-029</t>
+  </si>
+  <si>
+    <t>WC-2026-030</t>
+  </si>
+  <si>
+    <t>WC-2026-031</t>
+  </si>
+  <si>
+    <t>WC-2026-033</t>
+  </si>
+  <si>
+    <t>WC-2026-032</t>
+  </si>
+  <si>
+    <t>WC-2026-036</t>
+  </si>
+  <si>
+    <t>WC-2026-034</t>
+  </si>
+  <si>
+    <t>WC-2026-035</t>
+  </si>
+  <si>
+    <t>WC-2026-037</t>
+  </si>
+  <si>
+    <t>WC-2026-038</t>
+  </si>
+  <si>
+    <t>WC-2026-039</t>
+  </si>
+  <si>
+    <t>WC-2026-050</t>
+  </si>
+  <si>
+    <t>WC-2026-049</t>
+  </si>
+  <si>
+    <t>WC-2026-048</t>
+  </si>
+  <si>
+    <t>WC-2026-047</t>
+  </si>
+  <si>
+    <t>WC-2026-046</t>
+  </si>
+  <si>
+    <t>WC-2026-045</t>
+  </si>
+  <si>
+    <t>WC-2026-044</t>
+  </si>
+  <si>
+    <t>WC-2026-043</t>
+  </si>
+  <si>
+    <t>WC-2026-042</t>
+  </si>
+  <si>
+    <t>WC-2026-041</t>
+  </si>
+  <si>
+    <t>WC-2026-040</t>
+  </si>
+  <si>
+    <t>WC-2026-023</t>
+  </si>
+  <si>
+    <t>WC-2026-025</t>
+  </si>
+  <si>
+    <t>WC-2026-024</t>
+  </si>
+  <si>
+    <t>WC-2026-026</t>
+  </si>
+  <si>
+    <t>WC-2026-027</t>
+  </si>
+  <si>
+    <t>WC-2026-028</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>Bosnia and Herzegovina</t>
+  </si>
+  <si>
+    <t>Squad against Bosnia and Herzegovina</t>
+  </si>
+  <si>
+    <t>Squad against Canada</t>
+  </si>
+  <si>
+    <t>Maxime</t>
+  </si>
+  <si>
+    <t>Crepeau</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Maxime_Cr%C3%A9peau</t>
+  </si>
+  <si>
+    <t>Alistair</t>
+  </si>
+  <si>
+    <t>Johnston</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Alistair_Johnston</t>
+  </si>
+  <si>
+    <t>Luc</t>
+  </si>
+  <si>
+    <t>de Fougerolles</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Luc_de_Fougerolles</t>
+  </si>
+  <si>
+    <t>Derek</t>
+  </si>
+  <si>
+    <t>Cornelius</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Derek_Cornelius</t>
+  </si>
+  <si>
+    <t>Richie</t>
+  </si>
+  <si>
+    <t>Laryea</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Richie_Laryea</t>
+  </si>
+  <si>
+    <t>Tajon</t>
+  </si>
+  <si>
+    <t>Buchanan</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Tajon_Buchanan</t>
+  </si>
+  <si>
+    <t>Stephen</t>
+  </si>
+  <si>
+    <t>Eustaquio</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Stephen_Eust%C3%A1quio</t>
+  </si>
+  <si>
+    <t>Ismael</t>
+  </si>
+  <si>
+    <t>Kone</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Isma%C3%ABl_Kon%C3%A9</t>
+  </si>
+  <si>
+    <t>Liam</t>
+  </si>
+  <si>
+    <t>Millar</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Liam_Millar</t>
+  </si>
+  <si>
+    <t>Jonathan</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Jonathan_David</t>
+  </si>
+  <si>
+    <t>Cyle</t>
+  </si>
+  <si>
+    <t>Larin</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Cyle_Larin</t>
+  </si>
+  <si>
+    <t>Nikola</t>
+  </si>
+  <si>
+    <t>Vasilj</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Nikola_Vasilj</t>
+  </si>
+  <si>
+    <t>Tarik</t>
+  </si>
+  <si>
+    <t>Muharemovic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Tarik_Muharemovi%C4%87</t>
+  </si>
+  <si>
+    <t>Katic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Nikola_Kati%C4%87</t>
+  </si>
+  <si>
+    <t>Sead</t>
+  </si>
+  <si>
+    <t>Kolasinac</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Sead_Kola%C5%A1inac</t>
+  </si>
+  <si>
+    <t>Amar</t>
+  </si>
+  <si>
+    <t>Dedic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Amar_Dedi%C4%87</t>
+  </si>
+  <si>
+    <t>Ivan</t>
+  </si>
+  <si>
+    <t>Sunjic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ivan_%C5%A0unji%C4%87</t>
+  </si>
+  <si>
+    <t>Amir</t>
+  </si>
+  <si>
+    <t>Hadziahmetovic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Amir_Had%C5%BEiahmetovi%C4%87</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ivan_Ba%C5%A1i%C4%87</t>
+  </si>
+  <si>
+    <t>Esmir</t>
+  </si>
+  <si>
+    <t>Bajraktarevic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Esmir_Bajraktarevi%C4%87</t>
+  </si>
+  <si>
+    <t>Kerim</t>
+  </si>
+  <si>
+    <t>Alajbegovic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Kerim_Alajbegovi%C4%87</t>
+  </si>
+  <si>
+    <t>Ermedin</t>
+  </si>
+  <si>
+    <t>Demirovic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ermedin_Demirovi%C4%87</t>
+  </si>
+  <si>
+    <t>WC-2026-072</t>
+  </si>
+  <si>
+    <t>WC-2026-070</t>
+  </si>
+  <si>
+    <t>WC-2026-069</t>
+  </si>
+  <si>
+    <t>WC-2026-066</t>
+  </si>
+  <si>
+    <t>WC-2026-065</t>
+  </si>
+  <si>
+    <t>WC-2026-051</t>
+  </si>
+  <si>
+    <t>WC-2026-052</t>
+  </si>
+  <si>
+    <t>WC-2026-053</t>
+  </si>
+  <si>
+    <t>WC-2026-054</t>
+  </si>
+  <si>
+    <t>WC-2026-055</t>
+  </si>
+  <si>
+    <t>WC-2026-056</t>
+  </si>
+  <si>
+    <t>WC-2026-057</t>
+  </si>
+  <si>
+    <t>WC-2026-058</t>
+  </si>
+  <si>
+    <t>WC-2026-059</t>
+  </si>
+  <si>
+    <t>WC-2026-060</t>
+  </si>
+  <si>
+    <t>WC-2026-062</t>
+  </si>
+  <si>
+    <t>WC-2026-063</t>
+  </si>
+  <si>
+    <t>WC-2026-064</t>
+  </si>
+  <si>
+    <t>Tani</t>
+  </si>
+  <si>
+    <t>Oluwaseyi</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Tani_Oluwaseyi</t>
+  </si>
+  <si>
+    <t>WC-2026-073</t>
+  </si>
+  <si>
+    <t>Jovo</t>
+  </si>
+  <si>
+    <t>Lukic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Jovo_Luki%C4%87</t>
+  </si>
+  <si>
+    <t>Memic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Amar_Memi%C4%87</t>
+  </si>
+  <si>
+    <t>Benjamin</t>
+  </si>
+  <si>
+    <t>Tahirovic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Benjamin_Tahirovi%C4%87</t>
+  </si>
+  <si>
+    <t>WC-2026-076</t>
+  </si>
+  <si>
+    <t>WC-2026-075</t>
+  </si>
+  <si>
+    <t>WC-2026-074</t>
   </si>
 </sst>
 </file>
@@ -241,9 +998,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -265,6 +1022,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -283,22 +1054,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -336,9 +1117,6 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -356,9 +1134,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -373,8 +1148,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}" name="Table2" displayName="Table2" ref="A1:C3" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:C3" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}" name="Table2" displayName="Table2" ref="A1:C7" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:C7" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{112FDC7F-E515-4C7B-8F5E-37C3E12F8087}" name="ID"/>
     <tableColumn id="2" xr3:uid="{32773D89-5DDC-4032-9173-6B27222FCCB5}" name="Country"/>
@@ -385,19 +1160,21 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}" name="Table1" displayName="Table1" ref="A1:I23" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:I23" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}" name="Table1" displayName="Table1" ref="A1:K77" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:K77" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{4306409D-9EFE-4174-8717-966F7E42E287}" name="ID">
       <calculatedColumnFormula xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{7B72C7A7-BB87-4C46-9AEE-C1FCB4E8370C}" name="birth_date" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{F2C7799F-919A-4A78-B73F-0104748BDC42}" name="first_name"/>
+    <tableColumn id="11" xr3:uid="{3EE3FC3A-05D5-401C-9C1F-8AEADDCC8ED4}" name="last_name"/>
+    <tableColumn id="2" xr3:uid="{7B72C7A7-BB87-4C46-9AEE-C1FCB4E8370C}" name="birth_date" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{56118428-9B82-4DE8-B0E5-D3867A0971BB}" name="goalkeeper"/>
     <tableColumn id="4" xr3:uid="{63C03743-8698-49D0-B28F-811E3B1373E1}" name="defender"/>
     <tableColumn id="5" xr3:uid="{DC37E369-4FF2-4FC4-B514-796CECB10B1C}" name="midfielder"/>
     <tableColumn id="6" xr3:uid="{4DFCD6B3-8522-4468-9328-0D2A1C8A7CD3}" name="forward"/>
     <tableColumn id="7" xr3:uid="{F300BBF3-41B9-48EC-B798-A2D33A8B6F0A}" name="count_tournaments"/>
-    <tableColumn id="8" xr3:uid="{4AF02BFA-E31D-4884-BAF6-D352D492014A}" name="list_tournaments" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{4AF02BFA-E31D-4884-BAF6-D352D492014A}" name="list_tournaments" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{2ED820A1-163A-46C3-978A-E02F994BB2BA}" name="wikipedia"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -405,8 +1182,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}" name="Table3" displayName="Table3" ref="A1:B23" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B23" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}" name="Table3" displayName="Table3" ref="A1:B67" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:B67" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{397AF02E-7B1A-478B-BDCC-B7DFD6BA0DA4}" name="squad_id"/>
     <tableColumn id="2" xr3:uid="{CA2F8850-33A4-4388-8AFA-9498D25A5FA6}" name="player_id"/>
@@ -712,11 +1489,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB164D5D-EB26-4959-8B85-9C69F5946791}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -752,10 +1529,54 @@
         <v>6</v>
       </c>
     </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C6" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C7" t="s">
+        <v>223</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{4602E1B6-1F8E-4EA1-9981-FA346110476E}">
-      <formula1>"Mexico,South Africa"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{F89409D1-484E-49AE-8E6F-79B6E8003E5A}">
+      <formula1>"Mexico,South Africa, South Korea, Czech Republic, Canada, Bosnia and Herzegovina"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -768,245 +1589,289 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36DBA355-9A51-4754-A827-64470F21B097}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" customWidth="1"/>
-    <col min="6" max="6" width="9.5546875" customWidth="1"/>
-    <col min="7" max="7" width="19.6640625" customWidth="1"/>
-    <col min="8" max="8" width="49.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="65.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" customWidth="1"/>
+    <col min="9" max="9" width="19.6640625" customWidth="1"/>
+    <col min="10" max="10" width="49.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="72.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="str">
         <f xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</f>
         <v>WC-2026-001</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="4">
         <v>31241</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
         <v>7</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
-        <f t="shared" ref="A3:A24" si="0" xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</f>
+        <f t="shared" ref="A3:A66" si="0" xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</f>
         <v>WC-2026-002</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="4">
         <v>34561</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
         <v>3</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-003</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="4">
         <v>36090</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
         <v>2</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-004</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" s="4">
         <v>35485</v>
       </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
         <v>3</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-005</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="3">
         <v>36669</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>2</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-006</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="3">
         <v>36654</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
       <c r="E7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
         <v>2</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-007</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -1014,29 +1879,35 @@
       <c r="G8">
         <v>1</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-008</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="4">
         <v>37789</v>
       </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -1044,359 +1915,431 @@
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="I9" t="s">
+      <c r="K9" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-009</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D10" s="3">
         <v>36999</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
       <c r="E10">
         <v>0</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
         <v>2</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-010</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" s="3">
         <v>33363</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
         <v>4</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I11" t="s">
+      <c r="K11" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-011</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" s="3">
         <v>36045</v>
       </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
       <c r="E12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
         <v>3</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I12" t="s">
+      <c r="K12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-012</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="3">
         <v>33624</v>
       </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
       <c r="E13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
       <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
         <v>4</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-013</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="3">
         <v>34902</v>
       </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
         <v>3</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-014</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" s="3">
         <v>34815</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
         <v>4</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-015</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="3">
         <v>34964</v>
       </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
         <v>2</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I16" t="s">
+      <c r="K16" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-016</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" s="3">
         <v>38022</v>
       </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
       <c r="E17">
         <v>0</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>1</v>
-      </c>
-      <c r="H17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-017</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="3">
         <v>35454</v>
       </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
       <c r="E18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
         <v>3</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-018</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="3">
         <v>36222</v>
       </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
       <c r="E19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
         <v>2</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I19" t="s">
+      <c r="K19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-019</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
       <c r="E20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
         <v>4</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I20" t="s">
+      <c r="K20" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-020</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" s="3">
         <v>38283</v>
       </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
       <c r="E21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1404,85 +2347,2056 @@
       <c r="G21">
         <v>1</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="I21" t="s">
+      <c r="K21" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-021</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="3">
         <v>37128</v>
       </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
       <c r="E22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
         <v>2</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I22" t="s">
+      <c r="K22" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>WC-2026-022</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="3">
         <v>36772</v>
       </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
         <v>3</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I23" t="s">
+      <c r="K23" t="s">
         <v>42</v>
       </c>
     </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-023</v>
+      </c>
+      <c r="B24" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" t="s">
+        <v>109</v>
+      </c>
+      <c r="D24" s="3">
+        <v>36581</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-024</v>
+      </c>
+      <c r="B25" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" t="s">
+        <v>112</v>
+      </c>
+      <c r="D25" s="3">
+        <v>35513</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-025</v>
+      </c>
+      <c r="B26" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="3">
+        <v>35052</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K26" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-026</v>
+      </c>
+      <c r="B27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="3">
+        <v>37016</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>2</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K27" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-027</v>
+      </c>
+      <c r="B28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" t="s">
+        <v>121</v>
+      </c>
+      <c r="D28" s="3">
+        <v>38614</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>1</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-028</v>
+      </c>
+      <c r="B29" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29" s="3">
+        <v>38037</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>1</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K29" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-029</v>
+      </c>
+      <c r="B30" t="s">
+        <v>126</v>
+      </c>
+      <c r="C30" t="s">
+        <v>127</v>
+      </c>
+      <c r="D30" s="3">
+        <v>33146</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>4</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K30" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-030</v>
+      </c>
+      <c r="B31" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" t="s">
+        <v>130</v>
+      </c>
+      <c r="D31" s="3">
+        <v>37424</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-031</v>
+      </c>
+      <c r="B32" t="s">
+        <v>126</v>
+      </c>
+      <c r="C32" t="s">
+        <v>132</v>
+      </c>
+      <c r="D32" s="3">
+        <v>35384</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>3</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-032</v>
+      </c>
+      <c r="B33" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33" s="3">
+        <v>36714</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>2</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K33" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-033</v>
+      </c>
+      <c r="B34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="3">
+        <v>36134</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K34" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-034</v>
+      </c>
+      <c r="B35" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" t="s">
+        <v>140</v>
+      </c>
+      <c r="D35" s="3">
+        <v>35328</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <v>3</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K35" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-035</v>
+      </c>
+      <c r="B36" t="s">
+        <v>142</v>
+      </c>
+      <c r="C36" t="s">
+        <v>143</v>
+      </c>
+      <c r="D36" s="3">
+        <v>35506</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>2</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K36" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-036</v>
+      </c>
+      <c r="B37" t="s">
+        <v>129</v>
+      </c>
+      <c r="C37" t="s">
+        <v>145</v>
+      </c>
+      <c r="D37" s="3">
+        <v>37465</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-037</v>
+      </c>
+      <c r="B38" t="s">
+        <v>129</v>
+      </c>
+      <c r="C38" t="s">
+        <v>147</v>
+      </c>
+      <c r="D38" s="3">
+        <v>36941</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>2</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K38" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-038</v>
+      </c>
+      <c r="B39" t="s">
+        <v>149</v>
+      </c>
+      <c r="C39" t="s">
+        <v>150</v>
+      </c>
+      <c r="D39" s="3">
+        <v>33793</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>5</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="K39" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-039</v>
+      </c>
+      <c r="B40" t="s">
+        <v>129</v>
+      </c>
+      <c r="C40" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40" s="3">
+        <v>33826</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>3</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K40" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-040</v>
+      </c>
+      <c r="B41" t="s">
+        <v>155</v>
+      </c>
+      <c r="C41" t="s">
+        <v>156</v>
+      </c>
+      <c r="D41" s="3">
+        <v>36889</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <v>1</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K41" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-041</v>
+      </c>
+      <c r="B42" t="s">
+        <v>158</v>
+      </c>
+      <c r="C42" t="s">
+        <v>159</v>
+      </c>
+      <c r="D42" s="3">
+        <v>35088</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>3</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K42" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-042</v>
+      </c>
+      <c r="B43" t="s">
+        <v>161</v>
+      </c>
+      <c r="C43" t="s">
+        <v>162</v>
+      </c>
+      <c r="D43" s="3">
+        <v>35361</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K43" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-043</v>
+      </c>
+      <c r="B44" t="s">
+        <v>164</v>
+      </c>
+      <c r="C44" t="s">
+        <v>165</v>
+      </c>
+      <c r="D44" s="3">
+        <v>33836</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K44" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-044</v>
+      </c>
+      <c r="B45" t="s">
+        <v>167</v>
+      </c>
+      <c r="C45" t="s">
+        <v>168</v>
+      </c>
+      <c r="D45" s="3">
+        <v>37713</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>1</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>1</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K45" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-045</v>
+      </c>
+      <c r="B46" t="s">
+        <v>170</v>
+      </c>
+      <c r="C46" t="s">
+        <v>171</v>
+      </c>
+      <c r="D46" s="3">
+        <v>34757</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
+        <v>3</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K46" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-046</v>
+      </c>
+      <c r="B47" t="s">
+        <v>173</v>
+      </c>
+      <c r="C47" t="s">
+        <v>174</v>
+      </c>
+      <c r="D47" s="3">
+        <v>33838</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>3</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K47" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-047</v>
+      </c>
+      <c r="B48" t="s">
+        <v>176</v>
+      </c>
+      <c r="C48" t="s">
+        <v>177</v>
+      </c>
+      <c r="D48" s="3">
+        <v>36270</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>2</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K48" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-048</v>
+      </c>
+      <c r="B49" t="s">
+        <v>179</v>
+      </c>
+      <c r="C49" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" s="3">
+        <v>36554</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>1</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K49" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-049</v>
+      </c>
+      <c r="B50" t="s">
+        <v>182</v>
+      </c>
+      <c r="C50" t="s">
+        <v>183</v>
+      </c>
+      <c r="D50" s="3">
+        <v>37688</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50">
+        <v>0</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K50" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-050</v>
+      </c>
+      <c r="B51" t="s">
+        <v>185</v>
+      </c>
+      <c r="C51" t="s">
+        <v>186</v>
+      </c>
+      <c r="D51" s="3">
+        <v>36663</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K51" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-051</v>
+      </c>
+      <c r="B52" t="s">
+        <v>224</v>
+      </c>
+      <c r="C52" t="s">
+        <v>225</v>
+      </c>
+      <c r="D52" s="3">
+        <v>34465</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>3</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K52" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-052</v>
+      </c>
+      <c r="B53" t="s">
+        <v>227</v>
+      </c>
+      <c r="C53" t="s">
+        <v>228</v>
+      </c>
+      <c r="D53" s="3">
+        <v>36076</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53">
+        <v>2</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K53" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-053</v>
+      </c>
+      <c r="B54" t="s">
+        <v>230</v>
+      </c>
+      <c r="C54" t="s">
+        <v>231</v>
+      </c>
+      <c r="D54" s="3">
+        <v>38637</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>1</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>1</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K54" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-054</v>
+      </c>
+      <c r="B55" t="s">
+        <v>233</v>
+      </c>
+      <c r="C55" t="s">
+        <v>234</v>
+      </c>
+      <c r="D55" s="3">
+        <v>35759</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>3</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K55" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-055</v>
+      </c>
+      <c r="B56" t="s">
+        <v>236</v>
+      </c>
+      <c r="C56" t="s">
+        <v>237</v>
+      </c>
+      <c r="D56" s="3">
+        <v>34706</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>1</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>2</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K56" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-056</v>
+      </c>
+      <c r="B57" t="s">
+        <v>239</v>
+      </c>
+      <c r="C57" t="s">
+        <v>240</v>
+      </c>
+      <c r="D57" s="3">
+        <v>36199</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>1</v>
+      </c>
+      <c r="H57">
+        <v>1</v>
+      </c>
+      <c r="I57">
+        <v>2</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K57" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-057</v>
+      </c>
+      <c r="B58" t="s">
+        <v>242</v>
+      </c>
+      <c r="C58" t="s">
+        <v>243</v>
+      </c>
+      <c r="D58" s="3">
+        <v>35420</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>1</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>2</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K58" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-058</v>
+      </c>
+      <c r="B59" t="s">
+        <v>245</v>
+      </c>
+      <c r="C59" t="s">
+        <v>246</v>
+      </c>
+      <c r="D59" s="3">
+        <v>37423</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
+        <v>1</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
+        <v>2</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K59" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-059</v>
+      </c>
+      <c r="B60" t="s">
+        <v>248</v>
+      </c>
+      <c r="C60" t="s">
+        <v>249</v>
+      </c>
+      <c r="D60" s="3">
+        <v>36430</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60">
+        <v>1</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60">
+        <v>3</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-060</v>
+      </c>
+      <c r="B61" t="s">
+        <v>251</v>
+      </c>
+      <c r="C61" t="s">
+        <v>252</v>
+      </c>
+      <c r="D61" s="3">
+        <v>36539</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
+        <v>1</v>
+      </c>
+      <c r="I61">
+        <v>3</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K61" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-061</v>
+      </c>
+      <c r="B62" t="s">
+        <v>254</v>
+      </c>
+      <c r="C62" t="s">
+        <v>255</v>
+      </c>
+      <c r="D62" s="3">
+        <v>34806</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
+        <v>1</v>
+      </c>
+      <c r="I62">
+        <v>4</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K62" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-062</v>
+      </c>
+      <c r="B63" t="s">
+        <v>257</v>
+      </c>
+      <c r="C63" t="s">
+        <v>258</v>
+      </c>
+      <c r="D63" s="3">
+        <v>35035</v>
+      </c>
+      <c r="E63">
+        <v>1</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>2</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K63" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-063</v>
+      </c>
+      <c r="B64" t="s">
+        <v>260</v>
+      </c>
+      <c r="C64" t="s">
+        <v>261</v>
+      </c>
+      <c r="D64" s="3">
+        <v>37680</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>1</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>1</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K64" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-064</v>
+      </c>
+      <c r="B65" t="s">
+        <v>257</v>
+      </c>
+      <c r="C65" t="s">
+        <v>263</v>
+      </c>
+      <c r="D65" s="3">
+        <v>35348</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>1</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>1</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K65" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" t="str">
+        <f t="shared" si="0"/>
+        <v>WC-2026-065</v>
+      </c>
+      <c r="B66" t="s">
+        <v>265</v>
+      </c>
+      <c r="C66" t="s">
+        <v>266</v>
+      </c>
+      <c r="D66" s="3">
+        <v>34140</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>1</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
+        <v>4</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K66" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" t="str">
+        <f t="shared" ref="A67:A77" si="1" xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</f>
+        <v>WC-2026-066</v>
+      </c>
+      <c r="B67" t="s">
+        <v>268</v>
+      </c>
+      <c r="C67" t="s">
+        <v>269</v>
+      </c>
+      <c r="D67" s="3">
+        <v>37486</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>1</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67">
+        <v>2</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K67" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-067</v>
+      </c>
+      <c r="B68" t="s">
+        <v>271</v>
+      </c>
+      <c r="C68" t="s">
+        <v>272</v>
+      </c>
+      <c r="D68" s="3">
+        <v>35347</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68">
+        <v>1</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K68" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-068</v>
+      </c>
+      <c r="B69" t="s">
+        <v>274</v>
+      </c>
+      <c r="C69" t="s">
+        <v>275</v>
+      </c>
+      <c r="D69" s="3">
+        <v>35497</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>1</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>2</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K69" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-069</v>
+      </c>
+      <c r="B70" t="s">
+        <v>271</v>
+      </c>
+      <c r="C70" t="s">
+        <v>277</v>
+      </c>
+      <c r="D70" s="3">
+        <v>37376</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>1</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>1</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K70" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-070</v>
+      </c>
+      <c r="B71" t="s">
+        <v>279</v>
+      </c>
+      <c r="C71" t="s">
+        <v>280</v>
+      </c>
+      <c r="D71" s="3">
+        <v>38421</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>0</v>
+      </c>
+      <c r="G71">
+        <v>1</v>
+      </c>
+      <c r="H71">
+        <v>0</v>
+      </c>
+      <c r="I71">
+        <v>1</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K71" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-071</v>
+      </c>
+      <c r="B72" t="s">
+        <v>282</v>
+      </c>
+      <c r="C72" t="s">
+        <v>283</v>
+      </c>
+      <c r="D72" s="8">
+        <v>39346</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+      <c r="G72">
+        <v>1</v>
+      </c>
+      <c r="H72">
+        <v>0</v>
+      </c>
+      <c r="I72">
+        <v>1</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K72" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-072</v>
+      </c>
+      <c r="B73" t="s">
+        <v>285</v>
+      </c>
+      <c r="C73" t="s">
+        <v>286</v>
+      </c>
+      <c r="D73" s="3">
+        <v>35879</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>0</v>
+      </c>
+      <c r="G73">
+        <v>0</v>
+      </c>
+      <c r="H73">
+        <v>1</v>
+      </c>
+      <c r="I73">
+        <v>2</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K73" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-073</v>
+      </c>
+      <c r="B74" t="s">
+        <v>306</v>
+      </c>
+      <c r="C74" t="s">
+        <v>307</v>
+      </c>
+      <c r="D74" s="3">
+        <v>36661</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74">
+        <v>1</v>
+      </c>
+      <c r="I74">
+        <v>1</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K74" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-074</v>
+      </c>
+      <c r="B75" t="s">
+        <v>310</v>
+      </c>
+      <c r="C75" t="s">
+        <v>311</v>
+      </c>
+      <c r="D75" s="3">
+        <v>36127</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
+      </c>
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="I75">
+        <v>2</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K75" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-075</v>
+      </c>
+      <c r="B76" t="s">
+        <v>268</v>
+      </c>
+      <c r="C76" t="s">
+        <v>313</v>
+      </c>
+      <c r="D76" s="3">
+        <v>36911</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
+      </c>
+      <c r="G76">
+        <v>1</v>
+      </c>
+      <c r="H76">
+        <v>0</v>
+      </c>
+      <c r="I76">
+        <v>1</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K76" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-076</v>
+      </c>
+      <c r="B77" t="s">
+        <v>315</v>
+      </c>
+      <c r="C77" t="s">
+        <v>316</v>
+      </c>
+      <c r="D77" s="3">
+        <v>37683</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>1</v>
+      </c>
+      <c r="H77">
+        <v>0</v>
+      </c>
+      <c r="I77">
+        <v>1</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K77" t="s">
+        <v>317</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="K3" r:id="rId1" xr:uid="{E6C86540-6F11-4057-A81F-13C12F28CB53}"/>
+    <hyperlink ref="K5" r:id="rId2" xr:uid="{F873A396-A081-4C37-BDAD-E31AA41DEE6C}"/>
+    <hyperlink ref="K7" r:id="rId3" xr:uid="{5B928F3D-AF45-4D92-8C59-9FBE303C6EFA}"/>
+    <hyperlink ref="K8" r:id="rId4" xr:uid="{7A28B326-2A58-415E-8DB4-E3C30582A81D}"/>
+    <hyperlink ref="K9" r:id="rId5" xr:uid="{D0F6C453-770D-4372-ACFE-F8CC56C98149}"/>
+    <hyperlink ref="K11" r:id="rId6" xr:uid="{9A0847FD-9394-4F13-9C32-A6DCEB8EBDA4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4456234E-FBED-4764-8A48-D5C7CDF7A533}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -1502,7 +4416,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1510,7 +4424,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1518,7 +4432,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1526,7 +4440,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -1534,7 +4448,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1542,7 +4456,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -1550,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -1558,7 +4472,7 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -1566,7 +4480,7 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -1574,7 +4488,7 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -1582,7 +4496,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -1590,7 +4504,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -1598,7 +4512,7 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -1606,7 +4520,7 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -1614,7 +4528,7 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -1622,7 +4536,7 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -1630,7 +4544,7 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -1638,7 +4552,7 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -1646,7 +4560,7 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -1654,7 +4568,7 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>219</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -1662,7 +4576,7 @@
         <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -1670,7 +4584,359 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>3</v>
+      </c>
+      <c r="B26" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>3</v>
+      </c>
+      <c r="B27" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>3</v>
+      </c>
+      <c r="B30" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>3</v>
+      </c>
+      <c r="B31" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>3</v>
+      </c>
+      <c r="B32" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>4</v>
+      </c>
+      <c r="B42" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>4</v>
+      </c>
+      <c r="B43" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>4</v>
+      </c>
+      <c r="B44" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>4</v>
+      </c>
+      <c r="B45" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>5</v>
+      </c>
+      <c r="B46" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>5</v>
+      </c>
+      <c r="B47" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>5</v>
+      </c>
+      <c r="B48" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>5</v>
+      </c>
+      <c r="B49" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>5</v>
+      </c>
+      <c r="B50" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>5</v>
+      </c>
+      <c r="B51" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>5</v>
+      </c>
+      <c r="B52" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>5</v>
+      </c>
+      <c r="B53" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>5</v>
+      </c>
+      <c r="B54" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>5</v>
+      </c>
+      <c r="B55" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>5</v>
+      </c>
+      <c r="B56" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>6</v>
+      </c>
+      <c r="B57" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>6</v>
+      </c>
+      <c r="B58" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>6</v>
+      </c>
+      <c r="B59" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>6</v>
+      </c>
+      <c r="B60" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>6</v>
+      </c>
+      <c r="B61" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>6</v>
+      </c>
+      <c r="B62" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>6</v>
+      </c>
+      <c r="B63" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>6</v>
+      </c>
+      <c r="B64" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>6</v>
+      </c>
+      <c r="B65" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>6</v>
+      </c>
+      <c r="B66" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>6</v>
+      </c>
+      <c r="B67" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -1681,18 +4947,18 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{68D9C32C-35CC-4328-8038-1104A7225A69}">
+          <x14:formula1>
+            <xm:f>Players!$A:$A</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1:B1048576</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EC67924D-D32F-41C9-A4E6-B00ACDCC2077}">
           <x14:formula1>
             <xm:f>Squads!$A:$A</xm:f>
           </x14:formula1>
           <xm:sqref>A1:A1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{68D9C32C-35CC-4328-8038-1104A7225A69}">
-          <x14:formula1>
-            <xm:f>Players!$A:$A</xm:f>
-          </x14:formula1>
-          <xm:sqref>B1:B1048576</xm:sqref>
-        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
feat: Day 3 of world cup
</commit_message>
<xml_diff>
--- a/Projects/FIFACompetition/WorldCup2026/data/World Cup 2026.xlsx
+++ b/Projects/FIFACompetition/WorldCup2026/data/World Cup 2026.xlsx
@@ -8,10 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roman\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F76DCD-2F2C-43CE-A376-696E3435EFD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C0ADBA-0A04-4222-855F-462B7634B4FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="6216" activeTab="1" xr2:uid="{FA6ECF04-EE65-4057-9D05-B2AD136BFF74}"/>
-    <workbookView xWindow="11424" yWindow="6120" windowWidth="11712" windowHeight="6216" activeTab="2" xr2:uid="{2CE22ED6-905D-4770-8C84-A6921D1589AF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FA6ECF04-EE65-4057-9D05-B2AD136BFF74}"/>
   </bookViews>
   <sheets>
     <sheet name="Squads" sheetId="1" r:id="rId1"/>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="499">
   <si>
     <t>ID</t>
   </si>
@@ -991,6 +990,540 @@
   </si>
   <si>
     <t>WC-2026-074</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>Paraguay</t>
+  </si>
+  <si>
+    <t>Squad against Paraguay</t>
+  </si>
+  <si>
+    <t>Squad against USA</t>
+  </si>
+  <si>
+    <t>Matt</t>
+  </si>
+  <si>
+    <t>Freese</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Matt_Freese</t>
+  </si>
+  <si>
+    <t>Alex</t>
+  </si>
+  <si>
+    <t>Freeman</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Alex_Freeman</t>
+  </si>
+  <si>
+    <t>Miles</t>
+  </si>
+  <si>
+    <t>Robinson</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Miles_Robinson_(soccer)</t>
+  </si>
+  <si>
+    <t>Tim</t>
+  </si>
+  <si>
+    <t>Ream</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Tim_Ream</t>
+  </si>
+  <si>
+    <t>Antonee</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Antonee_Robinson</t>
+  </si>
+  <si>
+    <t>Sergino</t>
+  </si>
+  <si>
+    <t>Dest</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Sergi%C3%B1o_Dest</t>
+  </si>
+  <si>
+    <t>Tyler</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Tyler_Adams</t>
+  </si>
+  <si>
+    <t>Weston</t>
+  </si>
+  <si>
+    <t>McKennie</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Weston_McKennie</t>
+  </si>
+  <si>
+    <t>Malik</t>
+  </si>
+  <si>
+    <t>Tillman</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Malik_Tillman</t>
+  </si>
+  <si>
+    <t>Christian</t>
+  </si>
+  <si>
+    <t>Pulisic</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Christian_Pulisic</t>
+  </si>
+  <si>
+    <t>Folarin</t>
+  </si>
+  <si>
+    <t>Balogun</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Folarin_Balogun</t>
+  </si>
+  <si>
+    <t>Gatito</t>
+  </si>
+  <si>
+    <t>Fernandez</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Gatito_Fern%C3%A1ndez</t>
+  </si>
+  <si>
+    <t>Juan</t>
+  </si>
+  <si>
+    <t>Caceres</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Juan_Jos%C3%A9_C%C3%A1ceres</t>
+  </si>
+  <si>
+    <t>Gustavo</t>
+  </si>
+  <si>
+    <t>Gomez</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Gustavo_G%C3%B3mez</t>
+  </si>
+  <si>
+    <t>Omar</t>
+  </si>
+  <si>
+    <t>Alderete</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Omar_Alderete</t>
+  </si>
+  <si>
+    <t>Junior</t>
+  </si>
+  <si>
+    <t>Alonso</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/J%C3%BAnior_Alonso</t>
+  </si>
+  <si>
+    <t>Diego</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Diego_G%C3%B3mez_(Paraguayan_footballer)</t>
+  </si>
+  <si>
+    <t>Damain</t>
+  </si>
+  <si>
+    <t>Bobadilla</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Dami%C3%A1n_Bobadilla</t>
+  </si>
+  <si>
+    <t>Andres</t>
+  </si>
+  <si>
+    <t>Cubas</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Andr%C3%A9s_Cubas</t>
+  </si>
+  <si>
+    <t>Miguel</t>
+  </si>
+  <si>
+    <t>Almiron</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Miguel_Almir%C3%B3n</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Maur%C3%ADcio_(footballer,_born_2001)</t>
+  </si>
+  <si>
+    <t>Mauricio</t>
+  </si>
+  <si>
+    <t>Magalheaes</t>
+  </si>
+  <si>
+    <t>Antonio</t>
+  </si>
+  <si>
+    <t>Snabria</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Antonio_Sanabria</t>
+  </si>
+  <si>
+    <t>WC-2026-098</t>
+  </si>
+  <si>
+    <t>WC-2026-097</t>
+  </si>
+  <si>
+    <t>WC-2026-096</t>
+  </si>
+  <si>
+    <t>WC-2026-095</t>
+  </si>
+  <si>
+    <t>WC-2026-094</t>
+  </si>
+  <si>
+    <t>WC-2026-093</t>
+  </si>
+  <si>
+    <t>WC-2026-092</t>
+  </si>
+  <si>
+    <t>WC-2026-091</t>
+  </si>
+  <si>
+    <t>WC-2026-090</t>
+  </si>
+  <si>
+    <t>WC-2026-089</t>
+  </si>
+  <si>
+    <t>WC-2026-088</t>
+  </si>
+  <si>
+    <t>WC-2026-087</t>
+  </si>
+  <si>
+    <t>WC-2026-086</t>
+  </si>
+  <si>
+    <t>WC-2026-085</t>
+  </si>
+  <si>
+    <t>WC-2026-084</t>
+  </si>
+  <si>
+    <t>WC-2026-083</t>
+  </si>
+  <si>
+    <t>WC-2026-082</t>
+  </si>
+  <si>
+    <t>WC-2026-081</t>
+  </si>
+  <si>
+    <t>WC-2026-080</t>
+  </si>
+  <si>
+    <t>WC-2026-079</t>
+  </si>
+  <si>
+    <t>WC-2026-078</t>
+  </si>
+  <si>
+    <t>WC-2026-077</t>
+  </si>
+  <si>
+    <t>Qatar</t>
+  </si>
+  <si>
+    <t>Squad against Switzerland</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Squad against Qatar</t>
+  </si>
+  <si>
+    <t>Mahmud</t>
+  </si>
+  <si>
+    <t>Abunada</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Mahmud_Abunada</t>
+  </si>
+  <si>
+    <t>Homam</t>
+  </si>
+  <si>
+    <t>Ahmed</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Homam_Ahmed</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Pedro_Miguel_(footballer)</t>
+  </si>
+  <si>
+    <t>Boualem</t>
+  </si>
+  <si>
+    <t>Khoukhi</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Boualem_Khoukhi</t>
+  </si>
+  <si>
+    <t>Ayoub</t>
+  </si>
+  <si>
+    <t>Al-Oui</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ayoub_Al-Oui</t>
+  </si>
+  <si>
+    <t>Jassem</t>
+  </si>
+  <si>
+    <t>Gaber</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Jassem_Gaber</t>
+  </si>
+  <si>
+    <t>Fathy</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ahmed_Fathy_(Qatari_footballer)</t>
+  </si>
+  <si>
+    <t>Karim</t>
+  </si>
+  <si>
+    <t>Boudiaf</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Karim_Boudiaf</t>
+  </si>
+  <si>
+    <t>Akram</t>
+  </si>
+  <si>
+    <t>Afif</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Akram_Afif</t>
+  </si>
+  <si>
+    <t>Ali</t>
+  </si>
+  <si>
+    <t>Almoez</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Almoez_Ali</t>
+  </si>
+  <si>
+    <t>Edmilson</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Edmilson_Junior</t>
+  </si>
+  <si>
+    <t>Gregor</t>
+  </si>
+  <si>
+    <t>Kobel</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Gregor_Kobel</t>
+  </si>
+  <si>
+    <t>Silvan</t>
+  </si>
+  <si>
+    <t>Widmer</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Silvan_Widmer</t>
+  </si>
+  <si>
+    <t>Nico</t>
+  </si>
+  <si>
+    <t>Elvedi</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Nico_Elvedi</t>
+  </si>
+  <si>
+    <t>Manuel</t>
+  </si>
+  <si>
+    <t>Akanji</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Manuel_Akanji</t>
+  </si>
+  <si>
+    <t>Ricardo</t>
+  </si>
+  <si>
+    <t>Rodriguez</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Ricardo_Rodriguez_(footballer)</t>
+  </si>
+  <si>
+    <t>Remo</t>
+  </si>
+  <si>
+    <t>Freuler</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Remo_Freuler</t>
+  </si>
+  <si>
+    <t>Granit</t>
+  </si>
+  <si>
+    <t>Xhaka</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Granit_Xhaka</t>
+  </si>
+  <si>
+    <t>Dan</t>
+  </si>
+  <si>
+    <t>Ndoye</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Dan_Ndoye</t>
+  </si>
+  <si>
+    <t>Michel</t>
+  </si>
+  <si>
+    <t>Aebisher</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Michel_Aebischer</t>
+  </si>
+  <si>
+    <t>Manzambi</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Johan_Manzambi</t>
+  </si>
+  <si>
+    <t>Breel</t>
+  </si>
+  <si>
+    <t>Embolo</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/Breel_Embolo</t>
+  </si>
+  <si>
+    <t>WC-2026-120</t>
+  </si>
+  <si>
+    <t>WC-2026-119</t>
+  </si>
+  <si>
+    <t>WC-2026-118</t>
+  </si>
+  <si>
+    <t>WC-2026-117</t>
+  </si>
+  <si>
+    <t>WC-2026-116</t>
+  </si>
+  <si>
+    <t>WC-2026-115</t>
+  </si>
+  <si>
+    <t>WC-2026-114</t>
+  </si>
+  <si>
+    <t>WC-2026-113</t>
+  </si>
+  <si>
+    <t>WC-2026-112</t>
+  </si>
+  <si>
+    <t>WC-2026-111</t>
+  </si>
+  <si>
+    <t>WC-2026-110</t>
+  </si>
+  <si>
+    <t>WC-2026-109</t>
+  </si>
+  <si>
+    <t>WC-2026-108</t>
+  </si>
+  <si>
+    <t>WC-2026-107</t>
+  </si>
+  <si>
+    <t>WC-2026-106</t>
+  </si>
+  <si>
+    <t>WC-2026-105</t>
+  </si>
+  <si>
+    <t>WC-2026-104</t>
+  </si>
+  <si>
+    <t>WC-2026-103</t>
+  </si>
+  <si>
+    <t>WC-2026-102</t>
+  </si>
+  <si>
+    <t>WC-2026-101</t>
+  </si>
+  <si>
+    <t>WC-2026-100</t>
+  </si>
+  <si>
+    <t>WC-2026-099</t>
   </si>
 </sst>
 </file>
@@ -1075,12 +1608,6 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1117,6 +1644,12 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1148,8 +1681,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}" name="Table2" displayName="Table2" ref="A1:C7" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:C7" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}" name="Table2" displayName="Table2" ref="A1:C12" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:C12" xr:uid="{2363F4B3-9711-42EF-A57C-C89DB5FBD2CD}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{112FDC7F-E515-4C7B-8F5E-37C3E12F8087}" name="ID"/>
     <tableColumn id="2" xr3:uid="{32773D89-5DDC-4032-9173-6B27222FCCB5}" name="Country"/>
@@ -1160,21 +1693,21 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}" name="Table1" displayName="Table1" ref="A1:K77" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:K77" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}" name="Table1" displayName="Table1" ref="A1:K121" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:K121" xr:uid="{10AB2DDD-9499-4EDD-BBBD-B1510E490E13}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{4306409D-9EFE-4174-8717-966F7E42E287}" name="ID">
       <calculatedColumnFormula xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{F2C7799F-919A-4A78-B73F-0104748BDC42}" name="first_name"/>
     <tableColumn id="11" xr3:uid="{3EE3FC3A-05D5-401C-9C1F-8AEADDCC8ED4}" name="last_name"/>
-    <tableColumn id="2" xr3:uid="{7B72C7A7-BB87-4C46-9AEE-C1FCB4E8370C}" name="birth_date" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{7B72C7A7-BB87-4C46-9AEE-C1FCB4E8370C}" name="birth_date" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{56118428-9B82-4DE8-B0E5-D3867A0971BB}" name="goalkeeper"/>
     <tableColumn id="4" xr3:uid="{63C03743-8698-49D0-B28F-811E3B1373E1}" name="defender"/>
     <tableColumn id="5" xr3:uid="{DC37E369-4FF2-4FC4-B514-796CECB10B1C}" name="midfielder"/>
     <tableColumn id="6" xr3:uid="{4DFCD6B3-8522-4468-9328-0D2A1C8A7CD3}" name="forward"/>
     <tableColumn id="7" xr3:uid="{F300BBF3-41B9-48EC-B798-A2D33A8B6F0A}" name="count_tournaments"/>
-    <tableColumn id="8" xr3:uid="{4AF02BFA-E31D-4884-BAF6-D352D492014A}" name="list_tournaments" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{4AF02BFA-E31D-4884-BAF6-D352D492014A}" name="list_tournaments" dataDxfId="2"/>
     <tableColumn id="9" xr3:uid="{2ED820A1-163A-46C3-978A-E02F994BB2BA}" name="wikipedia"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1182,8 +1715,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}" name="Table3" displayName="Table3" ref="A1:B67" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:B67" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}" name="Table3" displayName="Table3" ref="A1:B111" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:B111" xr:uid="{85DA9C2E-819F-4246-8BCA-4FEE68F7A352}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{397AF02E-7B1A-478B-BDCC-B7DFD6BA0DA4}" name="squad_id"/>
     <tableColumn id="2" xr3:uid="{CA2F8850-33A4-4388-8AFA-9498D25A5FA6}" name="player_id"/>
@@ -1489,7 +2022,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB164D5D-EB26-4959-8B85-9C69F5946791}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
@@ -1573,12 +2106,56 @@
         <v>223</v>
       </c>
     </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>322</v>
+      </c>
+      <c r="C8" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>323</v>
+      </c>
+      <c r="C9" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>411</v>
+      </c>
+      <c r="C10" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>413</v>
+      </c>
+      <c r="C11" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>321</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{F89409D1-484E-49AE-8E6F-79B6E8003E5A}">
-      <formula1>"Mexico,South Africa, South Korea, Czech Republic, Canada, Bosnia and Herzegovina"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
@@ -1589,7 +2166,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36DBA355-9A51-4754-A827-64470F21B097}">
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
@@ -3982,7 +4559,7 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="str">
-        <f t="shared" ref="A67:A77" si="1" xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</f>
+        <f t="shared" ref="A67:A121" si="1" xml:space="preserve"> "WC-2026-" &amp; TEXT(ROW() - 1, "000")</f>
         <v>WC-2026-066</v>
       </c>
       <c r="B67" t="s">
@@ -4374,6 +4951,1590 @@
       </c>
       <c r="K77" t="s">
         <v>317</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-077</v>
+      </c>
+      <c r="B78" t="s">
+        <v>326</v>
+      </c>
+      <c r="C78" t="s">
+        <v>327</v>
+      </c>
+      <c r="D78" s="3">
+        <v>36040</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78">
+        <v>0</v>
+      </c>
+      <c r="I78">
+        <v>1</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K78" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-078</v>
+      </c>
+      <c r="B79" t="s">
+        <v>329</v>
+      </c>
+      <c r="C79" t="s">
+        <v>330</v>
+      </c>
+      <c r="D79" s="3">
+        <v>38208</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>1</v>
+      </c>
+      <c r="G79">
+        <v>0</v>
+      </c>
+      <c r="H79">
+        <v>0</v>
+      </c>
+      <c r="I79">
+        <v>1</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K79" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-079</v>
+      </c>
+      <c r="B80" t="s">
+        <v>332</v>
+      </c>
+      <c r="C80" t="s">
+        <v>333</v>
+      </c>
+      <c r="D80" s="3">
+        <v>35503</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>1</v>
+      </c>
+      <c r="G80">
+        <v>0</v>
+      </c>
+      <c r="H80">
+        <v>0</v>
+      </c>
+      <c r="I80">
+        <v>2</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K80" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-080</v>
+      </c>
+      <c r="B81" t="s">
+        <v>335</v>
+      </c>
+      <c r="C81" t="s">
+        <v>336</v>
+      </c>
+      <c r="D81" s="3">
+        <v>32055</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>1</v>
+      </c>
+      <c r="G81">
+        <v>0</v>
+      </c>
+      <c r="H81">
+        <v>0</v>
+      </c>
+      <c r="I81">
+        <v>5</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="K81" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-081</v>
+      </c>
+      <c r="B82" t="s">
+        <v>338</v>
+      </c>
+      <c r="C82" t="s">
+        <v>333</v>
+      </c>
+      <c r="D82" s="3">
+        <v>35650</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>1</v>
+      </c>
+      <c r="G82">
+        <v>0</v>
+      </c>
+      <c r="H82">
+        <v>0</v>
+      </c>
+      <c r="I82">
+        <v>3</v>
+      </c>
+      <c r="J82" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K82" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-082</v>
+      </c>
+      <c r="B83" t="s">
+        <v>340</v>
+      </c>
+      <c r="C83" t="s">
+        <v>341</v>
+      </c>
+      <c r="D83" s="3">
+        <v>36833</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>1</v>
+      </c>
+      <c r="G83">
+        <v>0</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>2</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K83" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-083</v>
+      </c>
+      <c r="B84" t="s">
+        <v>343</v>
+      </c>
+      <c r="C84" t="s">
+        <v>118</v>
+      </c>
+      <c r="D84" s="3">
+        <v>36205</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="G84">
+        <v>1</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+      <c r="I84">
+        <v>3</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K84" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-084</v>
+      </c>
+      <c r="B85" t="s">
+        <v>345</v>
+      </c>
+      <c r="C85" t="s">
+        <v>346</v>
+      </c>
+      <c r="D85" s="3">
+        <v>36035</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85">
+        <v>1</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+      <c r="I85">
+        <v>3</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K85" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-085</v>
+      </c>
+      <c r="B86" t="s">
+        <v>348</v>
+      </c>
+      <c r="C86" t="s">
+        <v>349</v>
+      </c>
+      <c r="D86" s="3">
+        <v>37404</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="G86">
+        <v>1</v>
+      </c>
+      <c r="H86">
+        <v>0</v>
+      </c>
+      <c r="I86">
+        <v>2</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K86" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-086</v>
+      </c>
+      <c r="B87" t="s">
+        <v>351</v>
+      </c>
+      <c r="C87" t="s">
+        <v>352</v>
+      </c>
+      <c r="D87" s="3">
+        <v>36056</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87">
+        <v>1</v>
+      </c>
+      <c r="H87">
+        <v>0</v>
+      </c>
+      <c r="I87">
+        <v>3</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K87" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-087</v>
+      </c>
+      <c r="B88" t="s">
+        <v>354</v>
+      </c>
+      <c r="C88" t="s">
+        <v>355</v>
+      </c>
+      <c r="D88" s="3">
+        <v>37075</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88">
+        <v>0</v>
+      </c>
+      <c r="H88">
+        <v>1</v>
+      </c>
+      <c r="I88">
+        <v>1</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K88" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-088</v>
+      </c>
+      <c r="B89" t="s">
+        <v>357</v>
+      </c>
+      <c r="C89" t="s">
+        <v>358</v>
+      </c>
+      <c r="D89" s="3">
+        <v>32231</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+      <c r="F89">
+        <v>0</v>
+      </c>
+      <c r="G89">
+        <v>0</v>
+      </c>
+      <c r="H89">
+        <v>0</v>
+      </c>
+      <c r="I89">
+        <v>4</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K89" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-089</v>
+      </c>
+      <c r="B90" t="s">
+        <v>360</v>
+      </c>
+      <c r="C90" t="s">
+        <v>361</v>
+      </c>
+      <c r="D90" s="3">
+        <v>36678</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+      <c r="G90">
+        <v>0</v>
+      </c>
+      <c r="H90">
+        <v>0</v>
+      </c>
+      <c r="I90">
+        <v>1</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K90" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-090</v>
+      </c>
+      <c r="B91" t="s">
+        <v>363</v>
+      </c>
+      <c r="C91" t="s">
+        <v>364</v>
+      </c>
+      <c r="D91" s="3">
+        <v>34095</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>1</v>
+      </c>
+      <c r="G91">
+        <v>0</v>
+      </c>
+      <c r="H91">
+        <v>0</v>
+      </c>
+      <c r="I91">
+        <v>4</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K91" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-091</v>
+      </c>
+      <c r="B92" t="s">
+        <v>366</v>
+      </c>
+      <c r="C92" t="s">
+        <v>367</v>
+      </c>
+      <c r="D92" s="3">
+        <v>35425</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+      <c r="G92">
+        <v>0</v>
+      </c>
+      <c r="H92">
+        <v>0</v>
+      </c>
+      <c r="I92">
+        <v>3</v>
+      </c>
+      <c r="J92" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K92" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-092</v>
+      </c>
+      <c r="B93" t="s">
+        <v>369</v>
+      </c>
+      <c r="C93" t="s">
+        <v>370</v>
+      </c>
+      <c r="D93" s="3">
+        <v>34009</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93">
+        <v>1</v>
+      </c>
+      <c r="G93">
+        <v>0</v>
+      </c>
+      <c r="H93">
+        <v>0</v>
+      </c>
+      <c r="I93">
+        <v>4</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K93" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-093</v>
+      </c>
+      <c r="B94" t="s">
+        <v>372</v>
+      </c>
+      <c r="C94" t="s">
+        <v>364</v>
+      </c>
+      <c r="D94" s="3">
+        <v>37707</v>
+      </c>
+      <c r="E94">
+        <v>0</v>
+      </c>
+      <c r="F94">
+        <v>0</v>
+      </c>
+      <c r="G94">
+        <v>1</v>
+      </c>
+      <c r="H94">
+        <v>0</v>
+      </c>
+      <c r="I94">
+        <v>2</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K94" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-094</v>
+      </c>
+      <c r="B95" t="s">
+        <v>374</v>
+      </c>
+      <c r="C95" t="s">
+        <v>375</v>
+      </c>
+      <c r="D95" s="3">
+        <v>37083</v>
+      </c>
+      <c r="E95">
+        <v>0</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+      <c r="G95">
+        <v>1</v>
+      </c>
+      <c r="H95">
+        <v>0</v>
+      </c>
+      <c r="I95">
+        <v>1</v>
+      </c>
+      <c r="J95" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K95" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A96" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-095</v>
+      </c>
+      <c r="B96" t="s">
+        <v>377</v>
+      </c>
+      <c r="C96" t="s">
+        <v>378</v>
+      </c>
+      <c r="D96" s="3">
+        <v>35196</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="G96">
+        <v>1</v>
+      </c>
+      <c r="H96">
+        <v>0</v>
+      </c>
+      <c r="I96">
+        <v>2</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K96" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-096</v>
+      </c>
+      <c r="B97" t="s">
+        <v>380</v>
+      </c>
+      <c r="C97" t="s">
+        <v>381</v>
+      </c>
+      <c r="D97" s="3">
+        <v>34375</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="G97">
+        <v>1</v>
+      </c>
+      <c r="H97">
+        <v>0</v>
+      </c>
+      <c r="I97">
+        <v>3</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K97" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-097</v>
+      </c>
+      <c r="B98" t="s">
+        <v>384</v>
+      </c>
+      <c r="C98" t="s">
+        <v>385</v>
+      </c>
+      <c r="D98" s="3">
+        <v>37064</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="G98">
+        <v>1</v>
+      </c>
+      <c r="H98">
+        <v>0</v>
+      </c>
+      <c r="I98">
+        <v>1</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K98" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-098</v>
+      </c>
+      <c r="B99" t="s">
+        <v>386</v>
+      </c>
+      <c r="C99" t="s">
+        <v>387</v>
+      </c>
+      <c r="D99" s="3">
+        <v>35128</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+      <c r="G99">
+        <v>0</v>
+      </c>
+      <c r="H99">
+        <v>1</v>
+      </c>
+      <c r="I99">
+        <v>4</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K99" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-099</v>
+      </c>
+      <c r="B100" t="s">
+        <v>415</v>
+      </c>
+      <c r="C100" t="s">
+        <v>416</v>
+      </c>
+      <c r="D100" s="3">
+        <v>36561</v>
+      </c>
+      <c r="E100">
+        <v>1</v>
+      </c>
+      <c r="F100">
+        <v>0</v>
+      </c>
+      <c r="G100">
+        <v>0</v>
+      </c>
+      <c r="H100">
+        <v>0</v>
+      </c>
+      <c r="I100">
+        <v>1</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K100" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A101" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>418</v>
+      </c>
+      <c r="C101" t="s">
+        <v>419</v>
+      </c>
+      <c r="D101" s="3">
+        <v>36397</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>1</v>
+      </c>
+      <c r="G101">
+        <v>0</v>
+      </c>
+      <c r="H101">
+        <v>0</v>
+      </c>
+      <c r="I101">
+        <v>2</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K101" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A102" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>421</v>
+      </c>
+      <c r="C102" t="s">
+        <v>380</v>
+      </c>
+      <c r="D102" s="3">
+        <v>33091</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>1</v>
+      </c>
+      <c r="G102">
+        <v>0</v>
+      </c>
+      <c r="H102">
+        <v>0</v>
+      </c>
+      <c r="I102">
+        <v>3</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K102" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>423</v>
+      </c>
+      <c r="C103" t="s">
+        <v>424</v>
+      </c>
+      <c r="D103" s="3">
+        <v>33063</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>1</v>
+      </c>
+      <c r="G103">
+        <v>0</v>
+      </c>
+      <c r="H103">
+        <v>0</v>
+      </c>
+      <c r="I103">
+        <v>4</v>
+      </c>
+      <c r="J103" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K103" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>426</v>
+      </c>
+      <c r="C104" t="s">
+        <v>427</v>
+      </c>
+      <c r="D104" s="3">
+        <v>38422</v>
+      </c>
+      <c r="E104">
+        <v>0</v>
+      </c>
+      <c r="F104">
+        <v>1</v>
+      </c>
+      <c r="G104">
+        <v>0</v>
+      </c>
+      <c r="H104">
+        <v>0</v>
+      </c>
+      <c r="I104">
+        <v>1</v>
+      </c>
+      <c r="J104" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K104" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A105" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>429</v>
+      </c>
+      <c r="C105" t="s">
+        <v>430</v>
+      </c>
+      <c r="D105" s="3">
+        <v>37307</v>
+      </c>
+      <c r="E105">
+        <v>0</v>
+      </c>
+      <c r="F105">
+        <v>0</v>
+      </c>
+      <c r="G105">
+        <v>1</v>
+      </c>
+      <c r="H105">
+        <v>0</v>
+      </c>
+      <c r="I105">
+        <v>1</v>
+      </c>
+      <c r="J105" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K105" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A106" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>419</v>
+      </c>
+      <c r="C106" t="s">
+        <v>432</v>
+      </c>
+      <c r="D106" s="3">
+        <v>33994</v>
+      </c>
+      <c r="E106">
+        <v>0</v>
+      </c>
+      <c r="F106">
+        <v>0</v>
+      </c>
+      <c r="G106">
+        <v>1</v>
+      </c>
+      <c r="H106">
+        <v>0</v>
+      </c>
+      <c r="I106">
+        <v>3</v>
+      </c>
+      <c r="J106" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K106" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A107" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>434</v>
+      </c>
+      <c r="C107" t="s">
+        <v>435</v>
+      </c>
+      <c r="D107" s="3">
+        <v>33132</v>
+      </c>
+      <c r="E107">
+        <v>0</v>
+      </c>
+      <c r="F107">
+        <v>0</v>
+      </c>
+      <c r="G107">
+        <v>1</v>
+      </c>
+      <c r="H107">
+        <v>0</v>
+      </c>
+      <c r="I107">
+        <v>4</v>
+      </c>
+      <c r="J107" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K107" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A108" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>437</v>
+      </c>
+      <c r="C108" t="s">
+        <v>438</v>
+      </c>
+      <c r="D108" s="3">
+        <v>35387</v>
+      </c>
+      <c r="E108">
+        <v>0</v>
+      </c>
+      <c r="F108">
+        <v>0</v>
+      </c>
+      <c r="G108">
+        <v>1</v>
+      </c>
+      <c r="H108">
+        <v>0</v>
+      </c>
+      <c r="I108">
+        <v>3</v>
+      </c>
+      <c r="J108" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K108" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A109" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>441</v>
+      </c>
+      <c r="C109" t="s">
+        <v>440</v>
+      </c>
+      <c r="D109" s="3">
+        <v>35296</v>
+      </c>
+      <c r="E109">
+        <v>0</v>
+      </c>
+      <c r="F109">
+        <v>0</v>
+      </c>
+      <c r="G109">
+        <v>0</v>
+      </c>
+      <c r="H109">
+        <v>1</v>
+      </c>
+      <c r="I109">
+        <v>3</v>
+      </c>
+      <c r="J109" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K109" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A110" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>443</v>
+      </c>
+      <c r="C110" t="s">
+        <v>369</v>
+      </c>
+      <c r="D110" s="3">
+        <v>34565</v>
+      </c>
+      <c r="E110">
+        <v>0</v>
+      </c>
+      <c r="F110">
+        <v>0</v>
+      </c>
+      <c r="G110">
+        <v>0</v>
+      </c>
+      <c r="H110">
+        <v>1</v>
+      </c>
+      <c r="I110">
+        <v>1</v>
+      </c>
+      <c r="J110" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K110" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A111" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>445</v>
+      </c>
+      <c r="C111" t="s">
+        <v>446</v>
+      </c>
+      <c r="D111" s="3">
+        <v>35770</v>
+      </c>
+      <c r="E111">
+        <v>1</v>
+      </c>
+      <c r="F111">
+        <v>0</v>
+      </c>
+      <c r="G111">
+        <v>0</v>
+      </c>
+      <c r="H111">
+        <v>0</v>
+      </c>
+      <c r="I111">
+        <v>2</v>
+      </c>
+      <c r="J111" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K111" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A112" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>448</v>
+      </c>
+      <c r="C112" t="s">
+        <v>449</v>
+      </c>
+      <c r="D112" s="3">
+        <v>34033</v>
+      </c>
+      <c r="E112">
+        <v>0</v>
+      </c>
+      <c r="F112">
+        <v>1</v>
+      </c>
+      <c r="G112">
+        <v>0</v>
+      </c>
+      <c r="H112">
+        <v>0</v>
+      </c>
+      <c r="I112">
+        <v>4</v>
+      </c>
+      <c r="J112" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K112" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>451</v>
+      </c>
+      <c r="C113" t="s">
+        <v>452</v>
+      </c>
+      <c r="D113" s="3">
+        <v>35338</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>1</v>
+      </c>
+      <c r="G113">
+        <v>0</v>
+      </c>
+      <c r="H113">
+        <v>0</v>
+      </c>
+      <c r="I113">
+        <v>3</v>
+      </c>
+      <c r="J113" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K113" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-113</v>
+      </c>
+      <c r="B114" t="s">
+        <v>454</v>
+      </c>
+      <c r="C114" t="s">
+        <v>455</v>
+      </c>
+      <c r="D114" s="3">
+        <v>34899</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+      <c r="F114">
+        <v>1</v>
+      </c>
+      <c r="G114">
+        <v>0</v>
+      </c>
+      <c r="H114">
+        <v>0</v>
+      </c>
+      <c r="I114">
+        <v>3</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K114" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>457</v>
+      </c>
+      <c r="C115" t="s">
+        <v>458</v>
+      </c>
+      <c r="D115" s="3">
+        <v>33841</v>
+      </c>
+      <c r="E115">
+        <v>0</v>
+      </c>
+      <c r="F115">
+        <v>1</v>
+      </c>
+      <c r="G115">
+        <v>0</v>
+      </c>
+      <c r="H115">
+        <v>0</v>
+      </c>
+      <c r="I115">
+        <v>4</v>
+      </c>
+      <c r="J115" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K115" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>460</v>
+      </c>
+      <c r="C116" t="s">
+        <v>461</v>
+      </c>
+      <c r="D116" s="3">
+        <v>33709</v>
+      </c>
+      <c r="E116">
+        <v>0</v>
+      </c>
+      <c r="F116">
+        <v>0</v>
+      </c>
+      <c r="G116">
+        <v>1</v>
+      </c>
+      <c r="H116">
+        <v>0</v>
+      </c>
+      <c r="I116">
+        <v>3</v>
+      </c>
+      <c r="J116" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K116" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>463</v>
+      </c>
+      <c r="C117" t="s">
+        <v>464</v>
+      </c>
+      <c r="D117" s="3">
+        <v>33874</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>0</v>
+      </c>
+      <c r="G117">
+        <v>1</v>
+      </c>
+      <c r="H117">
+        <v>0</v>
+      </c>
+      <c r="I117">
+        <v>4</v>
+      </c>
+      <c r="J117" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K117" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>466</v>
+      </c>
+      <c r="C118" t="s">
+        <v>467</v>
+      </c>
+      <c r="D118" s="3">
+        <v>36824</v>
+      </c>
+      <c r="E118">
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>0</v>
+      </c>
+      <c r="G118">
+        <v>1</v>
+      </c>
+      <c r="H118">
+        <v>0</v>
+      </c>
+      <c r="I118">
+        <v>2</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K118" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>469</v>
+      </c>
+      <c r="C119" t="s">
+        <v>470</v>
+      </c>
+      <c r="D119" s="3">
+        <v>35436</v>
+      </c>
+      <c r="E119">
+        <v>0</v>
+      </c>
+      <c r="F119">
+        <v>0</v>
+      </c>
+      <c r="G119">
+        <v>1</v>
+      </c>
+      <c r="H119">
+        <v>0</v>
+      </c>
+      <c r="I119">
+        <v>2</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K119" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>95</v>
+      </c>
+      <c r="C120" t="s">
+        <v>472</v>
+      </c>
+      <c r="D120" s="3">
+        <v>38639</v>
+      </c>
+      <c r="E120">
+        <v>0</v>
+      </c>
+      <c r="F120">
+        <v>0</v>
+      </c>
+      <c r="G120">
+        <v>1</v>
+      </c>
+      <c r="H120">
+        <v>0</v>
+      </c>
+      <c r="I120">
+        <v>1</v>
+      </c>
+      <c r="J120" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K120" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121" t="str">
+        <f t="shared" si="1"/>
+        <v>WC-2026-120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>474</v>
+      </c>
+      <c r="C121" t="s">
+        <v>475</v>
+      </c>
+      <c r="D121" s="3">
+        <v>35475</v>
+      </c>
+      <c r="E121">
+        <v>0</v>
+      </c>
+      <c r="F121">
+        <v>0</v>
+      </c>
+      <c r="G121">
+        <v>0</v>
+      </c>
+      <c r="H121">
+        <v>1</v>
+      </c>
+      <c r="I121">
+        <v>3</v>
+      </c>
+      <c r="J121" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K121" t="s">
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -4396,7 +6557,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4456234E-FBED-4764-8A48-D5C7CDF7A533}">
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B111"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" customWidth="1"/>
@@ -4937,6 +7098,358 @@
       </c>
       <c r="B67" t="s">
         <v>288</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>7</v>
+      </c>
+      <c r="B68" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>7</v>
+      </c>
+      <c r="B69" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>7</v>
+      </c>
+      <c r="B70" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>7</v>
+      </c>
+      <c r="B71" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>7</v>
+      </c>
+      <c r="B72" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>7</v>
+      </c>
+      <c r="B73" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>7</v>
+      </c>
+      <c r="B74" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>7</v>
+      </c>
+      <c r="B75" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>7</v>
+      </c>
+      <c r="B76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>7</v>
+      </c>
+      <c r="B77" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>7</v>
+      </c>
+      <c r="B78" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>8</v>
+      </c>
+      <c r="B79" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>8</v>
+      </c>
+      <c r="B80" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>8</v>
+      </c>
+      <c r="B81" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>8</v>
+      </c>
+      <c r="B82" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>8</v>
+      </c>
+      <c r="B83" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>8</v>
+      </c>
+      <c r="B84" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>8</v>
+      </c>
+      <c r="B85" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>8</v>
+      </c>
+      <c r="B86" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>8</v>
+      </c>
+      <c r="B87" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>8</v>
+      </c>
+      <c r="B88" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>8</v>
+      </c>
+      <c r="B89" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>9</v>
+      </c>
+      <c r="B90" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>9</v>
+      </c>
+      <c r="B91" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>9</v>
+      </c>
+      <c r="B92" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>9</v>
+      </c>
+      <c r="B93" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>9</v>
+      </c>
+      <c r="B94" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>9</v>
+      </c>
+      <c r="B95" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>9</v>
+      </c>
+      <c r="B96" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>9</v>
+      </c>
+      <c r="B97" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>9</v>
+      </c>
+      <c r="B98" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>9</v>
+      </c>
+      <c r="B99" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100">
+        <v>9</v>
+      </c>
+      <c r="B100" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101">
+        <v>10</v>
+      </c>
+      <c r="B101" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A102">
+        <v>10</v>
+      </c>
+      <c r="B102" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103">
+        <v>10</v>
+      </c>
+      <c r="B103" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104">
+        <v>10</v>
+      </c>
+      <c r="B104" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>10</v>
+      </c>
+      <c r="B105" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>10</v>
+      </c>
+      <c r="B106" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <v>10</v>
+      </c>
+      <c r="B107" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108">
+        <v>10</v>
+      </c>
+      <c r="B108" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109">
+        <v>10</v>
+      </c>
+      <c r="B109" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110">
+        <v>10</v>
+      </c>
+      <c r="B110" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111">
+        <v>10</v>
+      </c>
+      <c r="B111" t="s">
+        <v>477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>